<commit_message>
Updated client testing excel sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/Client_testing.xlsx
+++ b/src/test/resources/Client_testing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521759_cognizant_com/Documents/Desktop/synergia-automation/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521737\Projects\synergia-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{A87B3C4D-5450-46E7-9298-D3C31948196D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A70D48E-BCF7-4319-BFE7-1537E1CC2D61}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02BEEE9E-B5CC-4DF8-A575-FEB3C8C28951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{11E1AE38-0767-499E-BC28-D622838C415E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>username</t>
   </si>
@@ -71,7 +71,13 @@
     <t>"0123456789"</t>
   </si>
   <si>
-    <t>"123456789"</t>
+    <t>"1234567909"</t>
+  </si>
+  <si>
+    <t>"1234563789"</t>
+  </si>
+  <si>
+    <t>kashi@yahoo.com</t>
   </si>
 </sst>
 </file>
@@ -142,10 +148,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -519,10 +521,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>

</xml_diff>